<commit_message>
update formality and score results, remove per-prompt score files
</commit_message>
<xml_diff>
--- a/src/formality_results.xlsx
+++ b/src/formality_results.xlsx
@@ -31,12 +31,18 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -57,11 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -547,8 +554,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -571,8 +576,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -595,8 +598,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -843,8 +844,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -931,8 +930,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -955,8 +952,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1043,8 +1038,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1067,8 +1060,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1123,8 +1114,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1403,8 +1392,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1491,8 +1478,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1547,8 +1532,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1603,8 +1586,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1627,8 +1608,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1651,8 +1630,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1803,8 +1780,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1827,8 +1802,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2267,8 +2240,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2291,8 +2262,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2315,8 +2284,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2371,8 +2338,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2395,8 +2360,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2419,8 +2382,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2475,8 +2436,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2499,8 +2458,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2523,8 +2480,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2547,8 +2502,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2571,8 +2524,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2595,8 +2546,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2651,8 +2600,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2675,8 +2622,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2699,8 +2644,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2755,8 +2698,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2779,8 +2720,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2803,8 +2742,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2827,8 +2764,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2851,8 +2786,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2875,8 +2808,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2931,8 +2862,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2955,8 +2884,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2979,8 +2906,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3003,8 +2928,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3027,8 +2950,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3115,8 +3036,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3139,8 +3058,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3163,8 +3080,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3219,8 +3134,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3243,8 +3156,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3267,8 +3178,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3291,8 +3200,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3315,8 +3222,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3339,8 +3244,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3427,8 +3330,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3451,8 +3352,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3477,12 +3376,12 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>you, i</t>
+          <t>i, you</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>What is “them,” and what exactly do you want to set them straight about—Boston real estate investing (e. | , “Boston is overpriced / impossible to cash flow”), or something else entirely?  Also, what citation style do you want (APA/MLA/Chicago), and do you need only peer‑reviewed journal articles (no government/industry reports)?  Once you confirm, I’ll write a ≤1000‑word essay with **≥5 peer‑reviewed citations**.</t>
+          <t>To write the essay, I need one clarification: **who is “them,” and what claim(s) do you want to set them straight about?** (e. | )  In the meantime, here is a **≤1000-word essay** that “sets straight” a common bundle of misconceptions I hear in Boston investing circles in 2024—namely that **(1) high rates automatically mean Boston prices must fall sharply, (2) new supply will quickly fix affordability, and (3) office weakness implies the whole market is broken**—grounded in peer‑reviewed research. | The most rational stance is not a one-line prediction, but a segmented strategy: invest where supply constraints and enduring demand are strongest, and where you can add value without assuming heroic macro tailwinds.</t>
         </is>
       </c>
     </row>
@@ -3539,8 +3438,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3563,8 +3460,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3587,8 +3482,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3611,8 +3504,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3635,8 +3526,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3659,8 +3548,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3683,8 +3570,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3707,8 +3592,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3763,8 +3646,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3819,8 +3700,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3875,8 +3754,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3899,8 +3776,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3923,8 +3798,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3947,8 +3820,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3971,8 +3842,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3995,8 +3864,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4051,8 +3918,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4075,8 +3940,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4099,8 +3962,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4123,8 +3984,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4179,8 +4038,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4203,8 +4060,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4227,8 +4082,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4251,8 +4104,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4371,8 +4222,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4395,8 +4244,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4419,8 +4266,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4433,7 +4278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4514,7 +4359,6 @@
           <t>Technique</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Write</t>
@@ -4865,7 +4709,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Total A1</t>
@@ -5221,7 +5064,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Total A2</t>
@@ -5577,7 +5419,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Total A3</t>
@@ -5650,7 +5491,6 @@
           <t>Total Informal Essay</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>5</t>
@@ -5709,6 +5549,73 @@
       <c r="N18" t="inlineStr">
         <is>
           <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Avg Total Score</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>18.61</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>16.83</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>17.19</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>18.66</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>18.58</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>18.08</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>17.36</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>16.97</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>16.28</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>18.75</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>18.37</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>18.72</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5711,6 @@
           <t>Technique</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Write</t>
@@ -6510,7 +6416,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>1314</t>
         </is>
       </c>
     </row>

</xml_diff>